<commit_message>
Corriger des doublons de mapping et améliorer l'affichage e8d79281e87ab5c01f01a1250b9cf605f1ff27c3
</commit_message>
<xml_diff>
--- a/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
+++ b/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="116">
   <si>
     <t>Property</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-02T12:54:48+00:00</t>
+    <t>2026-09-02T15:48:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -257,6 +257,24 @@
     <t>ClinicalDocument.componentOf</t>
   </si>
   <si>
+    <t>FRLMHeaderDocument.documentReference</t>
+  </si>
+  <si>
+    <t>ClinicalDocument.relatedDocument</t>
+  </si>
+  <si>
+    <t>FRLMHeaderDocument.documentReference.relationType</t>
+  </si>
+  <si>
+    <t>RelatedDocument.typeCode</t>
+  </si>
+  <si>
+    <t>FRLMHeaderDocument.documentReference.targetDocument[x]</t>
+  </si>
+  <si>
+    <t>RelatedDocument.parentDocument</t>
+  </si>
+  <si>
     <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-bundle-document|0.1.0</t>
   </si>
   <si>
@@ -327,6 +345,27 @@
   </si>
   <si>
     <t>Composition.encounter</t>
+  </si>
+  <si>
+    <t>FRLMHeaderDocument.presentedForm</t>
+  </si>
+  <si>
+    <t>source-is-narrower-than-target</t>
+  </si>
+  <si>
+    <t>Composition.section</t>
+  </si>
+  <si>
+    <t>FRCompositionDocument.section:sectionAttachments ou FRCompositionDocument.section:sectionPresentedForm</t>
+  </si>
+  <si>
+    <t>Composition.relatesTo</t>
+  </si>
+  <si>
+    <t>Composition.relatesTo.code</t>
+  </si>
+  <si>
+    <t>Composition.relatesTo.target[x]</t>
   </si>
 </sst>
 </file>
@@ -582,7 +621,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -917,6 +956,45 @@
         <v>78</v>
       </c>
       <c r="E25" s="2"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D27" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D28" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="E28" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
@@ -956,7 +1034,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -971,7 +1049,7 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="E3" s="2"/>
     </row>
@@ -982,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1013,7 +1091,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -1028,7 +1106,7 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E3" s="2"/>
     </row>
@@ -1041,7 +1119,7 @@
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E4" s="2"/>
     </row>
@@ -1054,7 +1132,7 @@
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -1067,7 +1145,7 @@
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -1080,7 +1158,7 @@
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E7" s="2"/>
     </row>
@@ -1093,7 +1171,7 @@
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E8" s="2"/>
     </row>
@@ -1106,7 +1184,7 @@
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -1119,7 +1197,7 @@
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E10" s="2"/>
     </row>
@@ -1132,7 +1210,7 @@
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -1145,7 +1223,7 @@
         <v>34</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="E12" s="2"/>
     </row>
@@ -1158,7 +1236,7 @@
         <v>34</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E13" s="2"/>
     </row>
@@ -1171,7 +1249,7 @@
         <v>34</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E14" s="2"/>
     </row>
@@ -1184,7 +1262,7 @@
         <v>34</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E15" s="2"/>
     </row>
@@ -1197,7 +1275,7 @@
         <v>34</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="E16" s="2"/>
     </row>
@@ -1210,7 +1288,7 @@
         <v>34</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E17" s="2"/>
     </row>
@@ -1223,7 +1301,7 @@
         <v>34</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="E18" s="2"/>
     </row>
@@ -1236,7 +1314,7 @@
         <v>34</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E19" s="2"/>
     </row>
@@ -1249,7 +1327,7 @@
         <v>34</v>
       </c>
       <c r="D20" t="s" s="2">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E20" s="2"/>
     </row>
@@ -1262,7 +1340,7 @@
         <v>34</v>
       </c>
       <c r="D21" t="s" s="2">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="E21" s="2"/>
     </row>
@@ -1275,7 +1353,7 @@
         <v>34</v>
       </c>
       <c r="D22" t="s" s="2">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E22" s="2"/>
     </row>
@@ -1288,9 +1366,63 @@
         <v>34</v>
       </c>
       <c r="D23" t="s" s="2">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E23" s="2"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="D24" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="E24" t="s" s="2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D25" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D27" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="E27" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Ajouter une seconde cible pour presentedForm (extension diagnosticReport) e2e3cd1b5925216901268c2aadacf1cb007e3085
</commit_message>
<xml_diff>
--- a/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
+++ b/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="118">
   <si>
     <t>Property</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-02T15:48:56+00:00</t>
+    <t>2026-09-03T10:02:14+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -357,6 +357,12 @@
   </si>
   <si>
     <t>FRCompositionDocument.section:sectionAttachments ou FRCompositionDocument.section:sectionPresentedForm</t>
+  </si>
+  <si>
+    <t>Composition.extension</t>
+  </si>
+  <si>
+    <t>FRCompositionDocument.extension:diagnosticReport.presentedForm</t>
   </si>
   <si>
     <t>Composition.relatesTo</t>
@@ -1060,7 +1066,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1387,42 +1393,57 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>79</v>
+        <v>109</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" t="s" s="2">
-        <v>34</v>
+        <v>110</v>
       </c>
       <c r="D25" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="E25" s="2"/>
+      <c r="E25" t="s" s="2">
+        <v>114</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D26" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E26" s="2"/>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D27" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E27" s="2"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D28" t="s" s="2">
+        <v>117</v>
+      </c>
+      <c r="E28" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Restreindre la cible section de presentedForm à sectionPresentedForm 72fe3c8dbc96cd49b5e26f15c87105d10fde27e8
</commit_message>
<xml_diff>
--- a/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
+++ b/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-03T10:02:14+00:00</t>
+    <t>2026-09-03T10:35:28+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -356,7 +356,7 @@
     <t>Composition.section</t>
   </si>
   <si>
-    <t>FRCompositionDocument.section:sectionAttachments ou FRCompositionDocument.section:sectionPresentedForm</t>
+    <t>FRCompositionDocument.section:sectionPresentedForm</t>
   </si>
   <si>
     <t>Composition.extension</t>

</xml_diff>

<commit_message>
Référencer directement l'extension diagnosticReport pour presentedForm 1aff245d2e83bc358fd959102ce2a1d36399cfbb
</commit_message>
<xml_diff>
--- a/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
+++ b/fix-mapping-entete-duplicate-targets/ig/FRHeaderDocumentLMCDAFHIR.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="117">
   <si>
     <t>Property</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-03T10:35:28+00:00</t>
+    <t>2026-09-04T09:35:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -359,10 +359,7 @@
     <t>FRCompositionDocument.section:sectionPresentedForm</t>
   </si>
   <si>
-    <t>Composition.extension</t>
-  </si>
-  <si>
-    <t>FRCompositionDocument.extension:diagnosticReport.presentedForm</t>
+    <t>Composition.extension:diagnosticReport.presentedForm</t>
   </si>
   <si>
     <t>Composition.relatesTo</t>
@@ -1402,9 +1399,7 @@
       <c r="D25" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="E25" t="s" s="2">
-        <v>114</v>
-      </c>
+      <c r="E25" s="2"/>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
@@ -1415,7 +1410,7 @@
         <v>34</v>
       </c>
       <c r="D26" t="s" s="2">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E26" s="2"/>
     </row>
@@ -1428,7 +1423,7 @@
         <v>34</v>
       </c>
       <c r="D27" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E27" s="2"/>
     </row>
@@ -1441,7 +1436,7 @@
         <v>34</v>
       </c>
       <c r="D28" t="s" s="2">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E28" s="2"/>
     </row>

</xml_diff>